<commit_message>
chore(xlsx): BE v3 régénéré depuis v2 rempli (États en sortie + Catégorie d'état)
BE_prestations_v3.xlsx :
- 92 étapes avec États en sortie + dépendances préservés (saisies user v2)
- Colonne « Catégorie d'état » auto-mappée (51 EN_COURS / 24 EN_ATTENTE_RETOUR_ADMIN / 17 TERMINE)
- Onglet ÉTATS : 54 états (20 initiaux + 34 nouveaux détectés depuis les saisies)
  avec suggestion de catégorie macro par heuristique

scripts/_merge-v2-to-v3.mjs : nouveau script de fusion v2 → v3
.gitignore : ignore les fichiers de lock Excel ~$*

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BE_prestations_v2.xlsx
+++ b/BE_prestations_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\GITHUB\app_task\keon-outil-de-gestion-de-tache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FD208E-CC06-4EE9-A20C-0F79C7F619DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A12172-23BC-4B27-9BB5-21CDCFE23B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRESTATIONS" sheetId="1" r:id="rId1"/>

</xml_diff>